<commit_message>
Actualiza contenido y fotos
</commit_message>
<xml_diff>
--- a/plantilla_invitados_xv_sandra_alicia.xlsx
+++ b/plantilla_invitados_xv_sandra_alicia.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\XVSandra\xvsandra\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C499B1BA-24AA-4C4F-AE7A-2EAAD92BD490}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD1B3DAC-2531-40F7-B393-00EE288A46D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="177">
   <si>
     <t>codigo</t>
   </si>
@@ -217,9 +217,6 @@
     <t>Jesús y Wendy Montes</t>
   </si>
   <si>
-    <t>Oscar y Nelly  Villegas</t>
-  </si>
-  <si>
     <t>A004</t>
   </si>
   <si>
@@ -253,7 +250,322 @@
     <t>A014</t>
   </si>
   <si>
+    <t>A015</t>
+  </si>
+  <si>
+    <t>A016</t>
+  </si>
+  <si>
+    <t>A017</t>
+  </si>
+  <si>
+    <t>A018</t>
+  </si>
+  <si>
+    <t>A019</t>
+  </si>
+  <si>
+    <t>A020</t>
+  </si>
+  <si>
+    <t>A021</t>
+  </si>
+  <si>
+    <t>A022</t>
+  </si>
+  <si>
+    <t>A023</t>
+  </si>
+  <si>
+    <t>A024</t>
+  </si>
+  <si>
+    <t>A025</t>
+  </si>
+  <si>
+    <t>A026</t>
+  </si>
+  <si>
+    <t>A027</t>
+  </si>
+  <si>
+    <t>A028</t>
+  </si>
+  <si>
+    <t>A029</t>
+  </si>
+  <si>
+    <t>A030</t>
+  </si>
+  <si>
+    <t>A031</t>
+  </si>
+  <si>
+    <t>A032</t>
+  </si>
+  <si>
+    <t>A033</t>
+  </si>
+  <si>
+    <t>A034</t>
+  </si>
+  <si>
+    <t>A035</t>
+  </si>
+  <si>
+    <t>A036</t>
+  </si>
+  <si>
+    <t>A037</t>
+  </si>
+  <si>
+    <t>A038</t>
+  </si>
+  <si>
+    <t>A039</t>
+  </si>
+  <si>
+    <t>A040</t>
+  </si>
+  <si>
+    <t>A041</t>
+  </si>
+  <si>
+    <t>A042</t>
+  </si>
+  <si>
+    <t>A043</t>
+  </si>
+  <si>
+    <t>A044</t>
+  </si>
+  <si>
+    <t>A045</t>
+  </si>
+  <si>
+    <t>A046</t>
+  </si>
+  <si>
+    <t>A047</t>
+  </si>
+  <si>
+    <t>A048</t>
+  </si>
+  <si>
+    <t>A049</t>
+  </si>
+  <si>
+    <t>A050</t>
+  </si>
+  <si>
+    <t>A051</t>
+  </si>
+  <si>
+    <t>A052</t>
+  </si>
+  <si>
+    <t>A053</t>
+  </si>
+  <si>
+    <t>A054</t>
+  </si>
+  <si>
+    <t>A055</t>
+  </si>
+  <si>
+    <t>A056</t>
+  </si>
+  <si>
+    <t>A057</t>
+  </si>
+  <si>
+    <t>A058</t>
+  </si>
+  <si>
+    <t>A059</t>
+  </si>
+  <si>
+    <t>A060</t>
+  </si>
+  <si>
+    <t>A061</t>
+  </si>
+  <si>
+    <t>A062</t>
+  </si>
+  <si>
+    <t>A063</t>
+  </si>
+  <si>
+    <t>A064</t>
+  </si>
+  <si>
+    <t>A065</t>
+  </si>
+  <si>
     <t>https://xvsandra.vercel.app/</t>
+  </si>
+  <si>
+    <t>Columna1</t>
+  </si>
+  <si>
+    <t>https://xvsandra.vercel.app/?codigo=A009</t>
+  </si>
+  <si>
+    <t>Camila García</t>
+  </si>
+  <si>
+    <t>Ximena García</t>
+  </si>
+  <si>
+    <t>Dulce Villegas</t>
+  </si>
+  <si>
+    <t>Alexa Campos</t>
+  </si>
+  <si>
+    <t>Angela Martinéz</t>
+  </si>
+  <si>
+    <t>Vanessa Magaña</t>
+  </si>
+  <si>
+    <t>Yuliana García</t>
+  </si>
+  <si>
+    <t>Isabella Curiel</t>
+  </si>
+  <si>
+    <t>Isaac Jimenez</t>
+  </si>
+  <si>
+    <t>Salvador Vázquez</t>
+  </si>
+  <si>
+    <t>Daniel Alvarado</t>
+  </si>
+  <si>
+    <t>Estibaliz Vázquez</t>
+  </si>
+  <si>
+    <t>Daretzi Vázquez</t>
+  </si>
+  <si>
+    <t>Airam Vázquez</t>
+  </si>
+  <si>
+    <t>Yolanda Real</t>
+  </si>
+  <si>
+    <t>Jessica Amaya</t>
+  </si>
+  <si>
+    <t>Raymundo Felix</t>
+  </si>
+  <si>
+    <t>Matias Ibarra</t>
+  </si>
+  <si>
+    <t>Anna Julia</t>
+  </si>
+  <si>
+    <t>Violeth Correa</t>
+  </si>
+  <si>
+    <t>Gala Victoria</t>
+  </si>
+  <si>
+    <t>Sergio Muñoz</t>
+  </si>
+  <si>
+    <t>Ana Quintero</t>
+  </si>
+  <si>
+    <t>Emma Léon</t>
+  </si>
+  <si>
+    <t>Jimena Léon</t>
+  </si>
+  <si>
+    <t>Isabella Monroy</t>
+  </si>
+  <si>
+    <t>Monserrath Monroy</t>
+  </si>
+  <si>
+    <t>Maia Neri</t>
+  </si>
+  <si>
+    <t>Josue Quiroz</t>
+  </si>
+  <si>
+    <t>Paulina Ibarra</t>
+  </si>
+  <si>
+    <t>David Duarte</t>
+  </si>
+  <si>
+    <t>Lucia Sánchez</t>
+  </si>
+  <si>
+    <t>Lucia Nabor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dayana Vázquez </t>
+  </si>
+  <si>
+    <t>America Gonzalez</t>
+  </si>
+  <si>
+    <t>Dana López</t>
+  </si>
+  <si>
+    <t>Ashley Vásquez</t>
+  </si>
+  <si>
+    <t>Antonella Mártinez</t>
+  </si>
+  <si>
+    <t>Charlie Cardenas</t>
+  </si>
+  <si>
+    <t>Natalia Bojorquez</t>
+  </si>
+  <si>
+    <t>Myshelle Teran</t>
+  </si>
+  <si>
+    <t>Luna Villalobos</t>
+  </si>
+  <si>
+    <t>Camila Sánchez</t>
+  </si>
+  <si>
+    <t>Katherine Sánchez</t>
+  </si>
+  <si>
+    <t>Yadira Diaz</t>
+  </si>
+  <si>
+    <t>Sugey Diaz</t>
+  </si>
+  <si>
+    <t>Joel y Claudia Jimenez</t>
+  </si>
+  <si>
+    <t>Oscar y Nelly Villegas</t>
+  </si>
+  <si>
+    <t>Sandra A. Ruiz</t>
+  </si>
+  <si>
+    <t>Aleida Rojas</t>
+  </si>
+  <si>
+    <t>Veronica Cruz</t>
+  </si>
+  <si>
+    <t>Gonzalo y Silvia Rosales</t>
   </si>
 </sst>
 </file>
@@ -371,8 +683,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="InvitadosTable" displayName="InvitadosTable" ref="A1:G150">
-  <tableColumns count="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="InvitadosTable" displayName="InvitadosTable" ref="A1:H150">
+  <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="codigo"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="nombre"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="pases"/>
@@ -380,6 +692,7 @@
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="grupo"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="notas"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="link_invitacion"/>
+    <tableColumn id="8" xr3:uid="{2D05EE70-583D-4975-9CA1-AFED06FD5747}" name="Columna1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -534,7 +847,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G150"/>
+  <dimension ref="A1:H150"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -544,7 +857,7 @@
     <col min="7" max="7" width="48" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:8">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -566,16 +879,22 @@
       <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7">
+      <c r="H1" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>46</v>
+        <v>173</v>
       </c>
       <c r="C2">
         <v>2</v>
+      </c>
+      <c r="D2">
+        <v>6861159998</v>
       </c>
       <c r="E2" t="s">
         <v>47</v>
@@ -588,15 +907,18 @@
         <v>https://xvsandra.vercel.app/?codigo=A001</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:8">
       <c r="A3" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>6861138020</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3" t="str">
@@ -604,15 +926,18 @@
         <v>https://xvsandra.vercel.app/?codigo=A002</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:8">
       <c r="A4" s="3" t="s">
         <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C4">
-        <v>6</v>
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <v>6861876979</v>
       </c>
       <c r="F4" s="3"/>
       <c r="G4" s="3" t="str">
@@ -620,15 +945,18 @@
         <v>https://xvsandra.vercel.app/?codigo=A003</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:8">
       <c r="A5" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C5">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="D5">
+        <v>6861707740</v>
       </c>
       <c r="F5" s="3"/>
       <c r="G5" s="3" t="str">
@@ -636,15 +964,18 @@
         <v>https://xvsandra.vercel.app/?codigo=A004</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:8">
       <c r="A6" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C6">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="D6">
+        <v>6861575026</v>
       </c>
       <c r="F6" s="3"/>
       <c r="G6" s="3" t="str">
@@ -652,15 +983,18 @@
         <v>https://xvsandra.vercel.app/?codigo=A005</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:8">
       <c r="A7" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C7">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="D7">
+        <v>6866300023</v>
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="3" t="str">
@@ -668,15 +1002,18 @@
         <v>https://xvsandra.vercel.app/?codigo=A006</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:8">
       <c r="A8" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C8">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="D8">
+        <v>6863900811</v>
       </c>
       <c r="F8" s="3"/>
       <c r="G8" s="3" t="str">
@@ -684,31 +1021,40 @@
         <v>https://xvsandra.vercel.app/?codigo=A007</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:8">
       <c r="A9" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C9">
         <v>2</v>
+      </c>
+      <c r="D9">
+        <v>6862013354</v>
       </c>
       <c r="F9" s="3"/>
       <c r="G9" s="3" t="str">
         <f>IF(A9="","",Config!$B$2&amp;"?codigo="&amp;A9)</f>
         <v>https://xvsandra.vercel.app/?codigo=A008</v>
       </c>
-    </row>
-    <row r="10" spans="1:7">
+      <c r="H9" s="8" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
       <c r="A10" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C10">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="D10">
+        <v>6861084117</v>
       </c>
       <c r="F10" s="3"/>
       <c r="G10" s="3" t="str">
@@ -716,15 +1062,18 @@
         <v>https://xvsandra.vercel.app/?codigo=A009</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:8">
       <c r="A11" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C11">
         <v>1</v>
+      </c>
+      <c r="D11">
+        <v>6643567391</v>
       </c>
       <c r="F11" s="3"/>
       <c r="G11" s="3" t="str">
@@ -732,15 +1081,18 @@
         <v>https://xvsandra.vercel.app/?codigo=A010</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:8">
       <c r="A12" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B12" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C12">
         <v>1</v>
+      </c>
+      <c r="D12">
+        <v>6862485631</v>
       </c>
       <c r="F12" s="3"/>
       <c r="G12" s="3" t="str">
@@ -748,15 +1100,18 @@
         <v>https://xvsandra.vercel.app/?codigo=A011</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:8">
       <c r="A13" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C13">
         <v>1</v>
+      </c>
+      <c r="D13">
+        <v>6862412292</v>
       </c>
       <c r="F13" s="3"/>
       <c r="G13" s="3" t="str">
@@ -764,15 +1119,18 @@
         <v>https://xvsandra.vercel.app/?codigo=A012</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:8">
       <c r="A14" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B14" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C14">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="D14">
+        <v>6862434748</v>
       </c>
       <c r="F14" s="3"/>
       <c r="G14" s="3" t="str">
@@ -780,15 +1138,18 @@
         <v>https://xvsandra.vercel.app/?codigo=A013</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:8">
       <c r="A15" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B15" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C15">
         <v>2</v>
+      </c>
+      <c r="D15">
+        <v>6863150447</v>
       </c>
       <c r="F15" s="3"/>
       <c r="G15" s="3" t="str">
@@ -796,622 +1157,934 @@
         <v>https://xvsandra.vercel.app/?codigo=A014</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="3"/>
+    <row r="16" spans="1:8">
+      <c r="A16" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B16" t="s">
+        <v>172</v>
+      </c>
+      <c r="C16">
+        <v>2</v>
+      </c>
+      <c r="D16" s="3">
+        <v>6862710014</v>
+      </c>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
       <c r="G16" s="3" t="str">
         <f>IF(A16="","",Config!$B$2&amp;"?codigo="&amp;A16)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A015</v>
       </c>
     </row>
     <row r="17" spans="1:7">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="3"/>
+      <c r="A17" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B17" t="s">
+        <v>171</v>
+      </c>
+      <c r="C17">
+        <v>2</v>
+      </c>
+      <c r="D17" s="3">
+        <v>6869462795</v>
+      </c>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
       <c r="G17" s="3" t="str">
         <f>IF(A17="","",Config!$B$2&amp;"?codigo="&amp;A17)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A016</v>
       </c>
     </row>
     <row r="18" spans="1:7">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="3"/>
+      <c r="A18" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B18" t="s">
+        <v>174</v>
+      </c>
+      <c r="C18">
+        <v>2</v>
+      </c>
+      <c r="D18" s="3">
+        <v>6861634661</v>
+      </c>
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
       <c r="G18" s="3" t="str">
         <f>IF(A18="","",Config!$B$2&amp;"?codigo="&amp;A18)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A017</v>
       </c>
     </row>
     <row r="19" spans="1:7">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="3"/>
+      <c r="A19" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B19" t="s">
+        <v>175</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
+      <c r="D19" s="3">
+        <v>6861858868</v>
+      </c>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
       <c r="G19" s="3" t="str">
         <f>IF(A19="","",Config!$B$2&amp;"?codigo="&amp;A19)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A018</v>
       </c>
     </row>
     <row r="20" spans="1:7">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
-      <c r="C20" s="5"/>
+      <c r="A20" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B20" t="s">
+        <v>176</v>
+      </c>
+      <c r="C20">
+        <v>2</v>
+      </c>
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3" t="str">
         <f>IF(A20="","",Config!$B$2&amp;"?codigo="&amp;A20)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A019</v>
       </c>
     </row>
     <row r="21" spans="1:7">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
-      <c r="C21" s="5"/>
+      <c r="A21" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C21" s="5">
+        <v>1</v>
+      </c>
       <c r="D21" s="3"/>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3" t="str">
         <f>IF(A21="","",Config!$B$2&amp;"?codigo="&amp;A21)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A020</v>
       </c>
     </row>
     <row r="22" spans="1:7">
-      <c r="A22" s="3"/>
-      <c r="B22" s="3"/>
-      <c r="C22" s="5"/>
+      <c r="A22" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="C22" s="5">
+        <v>1</v>
+      </c>
       <c r="D22" s="3"/>
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
       <c r="G22" s="3" t="str">
         <f>IF(A22="","",Config!$B$2&amp;"?codigo="&amp;A22)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A021</v>
       </c>
     </row>
     <row r="23" spans="1:7">
-      <c r="A23" s="3"/>
-      <c r="B23" s="3"/>
-      <c r="C23" s="5"/>
+      <c r="A23" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C23" s="5">
+        <v>1</v>
+      </c>
       <c r="D23" s="3"/>
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
       <c r="G23" s="3" t="str">
         <f>IF(A23="","",Config!$B$2&amp;"?codigo="&amp;A23)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A022</v>
       </c>
     </row>
     <row r="24" spans="1:7">
-      <c r="A24" s="3"/>
-      <c r="B24" s="3"/>
-      <c r="C24" s="5"/>
+      <c r="A24" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C24" s="5">
+        <v>1</v>
+      </c>
       <c r="D24" s="3"/>
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
       <c r="G24" s="3" t="str">
         <f>IF(A24="","",Config!$B$2&amp;"?codigo="&amp;A24)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A023</v>
       </c>
     </row>
     <row r="25" spans="1:7">
-      <c r="A25" s="3"/>
-      <c r="B25" s="3"/>
-      <c r="C25" s="5"/>
+      <c r="A25" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C25" s="5">
+        <v>1</v>
+      </c>
       <c r="D25" s="3"/>
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
       <c r="G25" s="3" t="str">
         <f>IF(A25="","",Config!$B$2&amp;"?codigo="&amp;A25)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A024</v>
       </c>
     </row>
     <row r="26" spans="1:7">
-      <c r="A26" s="3"/>
-      <c r="B26" s="3"/>
-      <c r="C26" s="5"/>
+      <c r="A26" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C26" s="5">
+        <v>1</v>
+      </c>
       <c r="D26" s="3"/>
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
       <c r="G26" s="3" t="str">
         <f>IF(A26="","",Config!$B$2&amp;"?codigo="&amp;A26)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A025</v>
       </c>
     </row>
     <row r="27" spans="1:7">
-      <c r="A27" s="3"/>
-      <c r="B27" s="3"/>
-      <c r="C27" s="5"/>
+      <c r="A27" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C27" s="5">
+        <v>1</v>
+      </c>
       <c r="D27" s="3"/>
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
       <c r="G27" s="3" t="str">
         <f>IF(A27="","",Config!$B$2&amp;"?codigo="&amp;A27)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A026</v>
       </c>
     </row>
     <row r="28" spans="1:7">
-      <c r="A28" s="3"/>
-      <c r="B28" s="3"/>
-      <c r="C28" s="5"/>
+      <c r="A28" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C28" s="5">
+        <v>1</v>
+      </c>
       <c r="D28" s="3"/>
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
       <c r="G28" s="3" t="str">
         <f>IF(A28="","",Config!$B$2&amp;"?codigo="&amp;A28)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A027</v>
       </c>
     </row>
     <row r="29" spans="1:7">
-      <c r="A29" s="3"/>
-      <c r="B29" s="3"/>
-      <c r="C29" s="5"/>
+      <c r="A29" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="C29" s="5">
+        <v>1</v>
+      </c>
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>
       <c r="F29" s="3"/>
       <c r="G29" s="3" t="str">
         <f>IF(A29="","",Config!$B$2&amp;"?codigo="&amp;A29)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A028</v>
       </c>
     </row>
     <row r="30" spans="1:7">
-      <c r="A30" s="3"/>
-      <c r="B30" s="3"/>
-      <c r="C30" s="5"/>
+      <c r="A30" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="C30" s="5">
+        <v>1</v>
+      </c>
       <c r="D30" s="3"/>
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
       <c r="G30" s="3" t="str">
         <f>IF(A30="","",Config!$B$2&amp;"?codigo="&amp;A30)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A029</v>
       </c>
     </row>
     <row r="31" spans="1:7">
-      <c r="A31" s="3"/>
-      <c r="B31" s="3"/>
-      <c r="C31" s="5"/>
+      <c r="A31" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="C31" s="5">
+        <v>1</v>
+      </c>
       <c r="D31" s="3"/>
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
       <c r="G31" s="3" t="str">
         <f>IF(A31="","",Config!$B$2&amp;"?codigo="&amp;A31)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A030</v>
       </c>
     </row>
     <row r="32" spans="1:7">
-      <c r="A32" s="3"/>
-      <c r="B32" s="3"/>
-      <c r="C32" s="5"/>
+      <c r="A32" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="C32" s="5">
+        <v>1</v>
+      </c>
       <c r="D32" s="3"/>
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
       <c r="G32" s="3" t="str">
         <f>IF(A32="","",Config!$B$2&amp;"?codigo="&amp;A32)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A031</v>
       </c>
     </row>
     <row r="33" spans="1:7">
-      <c r="A33" s="3"/>
-      <c r="B33" s="3"/>
-      <c r="C33" s="5"/>
+      <c r="A33" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="C33" s="5">
+        <v>1</v>
+      </c>
       <c r="D33" s="3"/>
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
       <c r="G33" s="3" t="str">
         <f>IF(A33="","",Config!$B$2&amp;"?codigo="&amp;A33)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A032</v>
       </c>
     </row>
     <row r="34" spans="1:7">
-      <c r="A34" s="3"/>
-      <c r="B34" s="3"/>
-      <c r="C34" s="5"/>
+      <c r="A34" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="C34" s="5">
+        <v>1</v>
+      </c>
       <c r="D34" s="3"/>
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
       <c r="G34" s="3" t="str">
         <f>IF(A34="","",Config!$B$2&amp;"?codigo="&amp;A34)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A033</v>
       </c>
     </row>
     <row r="35" spans="1:7">
-      <c r="A35" s="3"/>
-      <c r="B35" s="3"/>
-      <c r="C35" s="5"/>
+      <c r="A35" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="C35" s="5">
+        <v>1</v>
+      </c>
       <c r="D35" s="3"/>
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
       <c r="G35" s="3" t="str">
         <f>IF(A35="","",Config!$B$2&amp;"?codigo="&amp;A35)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A034</v>
       </c>
     </row>
     <row r="36" spans="1:7">
-      <c r="A36" s="3"/>
-      <c r="B36" s="3"/>
-      <c r="C36" s="5"/>
+      <c r="A36" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="C36" s="5">
+        <v>1</v>
+      </c>
       <c r="D36" s="3"/>
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
       <c r="G36" s="3" t="str">
         <f>IF(A36="","",Config!$B$2&amp;"?codigo="&amp;A36)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A035</v>
       </c>
     </row>
     <row r="37" spans="1:7">
-      <c r="A37" s="3"/>
-      <c r="B37" s="3"/>
-      <c r="C37" s="5"/>
+      <c r="A37" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="C37" s="5">
+        <v>1</v>
+      </c>
       <c r="D37" s="3"/>
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
       <c r="G37" s="3" t="str">
         <f>IF(A37="","",Config!$B$2&amp;"?codigo="&amp;A37)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A036</v>
       </c>
     </row>
     <row r="38" spans="1:7">
-      <c r="A38" s="3"/>
-      <c r="B38" s="3"/>
-      <c r="C38" s="5"/>
+      <c r="A38" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="C38" s="5">
+        <v>1</v>
+      </c>
       <c r="D38" s="3"/>
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
       <c r="G38" s="3" t="str">
         <f>IF(A38="","",Config!$B$2&amp;"?codigo="&amp;A38)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A037</v>
       </c>
     </row>
     <row r="39" spans="1:7">
-      <c r="A39" s="3"/>
-      <c r="B39" s="3"/>
-      <c r="C39" s="5"/>
+      <c r="A39" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="C39" s="5">
+        <v>1</v>
+      </c>
       <c r="D39" s="3"/>
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
       <c r="G39" s="3" t="str">
         <f>IF(A39="","",Config!$B$2&amp;"?codigo="&amp;A39)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A038</v>
       </c>
     </row>
     <row r="40" spans="1:7">
-      <c r="A40" s="3"/>
-      <c r="B40" s="3"/>
-      <c r="C40" s="5"/>
+      <c r="A40" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="C40" s="5">
+        <v>1</v>
+      </c>
       <c r="D40" s="3"/>
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
       <c r="G40" s="3" t="str">
         <f>IF(A40="","",Config!$B$2&amp;"?codigo="&amp;A40)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A039</v>
       </c>
     </row>
     <row r="41" spans="1:7">
-      <c r="A41" s="3"/>
-      <c r="B41" s="3"/>
-      <c r="C41" s="5"/>
+      <c r="A41" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="C41" s="5">
+        <v>1</v>
+      </c>
       <c r="D41" s="3"/>
       <c r="E41" s="3"/>
       <c r="F41" s="3"/>
       <c r="G41" s="3" t="str">
         <f>IF(A41="","",Config!$B$2&amp;"?codigo="&amp;A41)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A040</v>
       </c>
     </row>
     <row r="42" spans="1:7">
-      <c r="A42" s="3"/>
-      <c r="B42" s="3"/>
-      <c r="C42" s="5"/>
+      <c r="A42" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="C42" s="5">
+        <v>1</v>
+      </c>
       <c r="D42" s="3"/>
       <c r="E42" s="3"/>
       <c r="F42" s="3"/>
       <c r="G42" s="3" t="str">
         <f>IF(A42="","",Config!$B$2&amp;"?codigo="&amp;A42)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A041</v>
       </c>
     </row>
     <row r="43" spans="1:7">
-      <c r="A43" s="3"/>
-      <c r="B43" s="3"/>
-      <c r="C43" s="5"/>
+      <c r="A43" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="C43" s="5">
+        <v>2</v>
+      </c>
       <c r="D43" s="3"/>
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
       <c r="G43" s="3" t="str">
         <f>IF(A43="","",Config!$B$2&amp;"?codigo="&amp;A43)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A042</v>
       </c>
     </row>
     <row r="44" spans="1:7">
-      <c r="A44" s="3"/>
-      <c r="B44" s="3"/>
-      <c r="C44" s="5"/>
+      <c r="A44" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="C44" s="5">
+        <v>1</v>
+      </c>
       <c r="D44" s="3"/>
       <c r="E44" s="3"/>
       <c r="F44" s="3"/>
       <c r="G44" s="3" t="str">
         <f>IF(A44="","",Config!$B$2&amp;"?codigo="&amp;A44)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A043</v>
       </c>
     </row>
     <row r="45" spans="1:7">
-      <c r="A45" s="3"/>
-      <c r="B45" s="3"/>
-      <c r="C45" s="5"/>
+      <c r="A45" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="C45" s="5">
+        <v>1</v>
+      </c>
       <c r="D45" s="3"/>
       <c r="E45" s="3"/>
       <c r="F45" s="3"/>
       <c r="G45" s="3" t="str">
         <f>IF(A45="","",Config!$B$2&amp;"?codigo="&amp;A45)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A044</v>
       </c>
     </row>
     <row r="46" spans="1:7">
-      <c r="A46" s="3"/>
-      <c r="B46" s="3"/>
-      <c r="C46" s="5"/>
+      <c r="A46" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="C46" s="5">
+        <v>1</v>
+      </c>
       <c r="D46" s="3"/>
       <c r="E46" s="3"/>
       <c r="F46" s="3"/>
       <c r="G46" s="3" t="str">
         <f>IF(A46="","",Config!$B$2&amp;"?codigo="&amp;A46)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A045</v>
       </c>
     </row>
     <row r="47" spans="1:7">
-      <c r="A47" s="3"/>
-      <c r="B47" s="3"/>
-      <c r="C47" s="5"/>
+      <c r="A47" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="C47" s="5">
+        <v>1</v>
+      </c>
       <c r="D47" s="3"/>
       <c r="E47" s="3"/>
       <c r="F47" s="3"/>
       <c r="G47" s="3" t="str">
         <f>IF(A47="","",Config!$B$2&amp;"?codigo="&amp;A47)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A046</v>
       </c>
     </row>
     <row r="48" spans="1:7">
-      <c r="A48" s="3"/>
-      <c r="B48" s="3"/>
-      <c r="C48" s="5"/>
+      <c r="A48" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C48" s="5">
+        <v>1</v>
+      </c>
       <c r="D48" s="3"/>
       <c r="E48" s="3"/>
       <c r="F48" s="3"/>
       <c r="G48" s="3" t="str">
         <f>IF(A48="","",Config!$B$2&amp;"?codigo="&amp;A48)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A047</v>
       </c>
     </row>
     <row r="49" spans="1:7">
-      <c r="A49" s="3"/>
-      <c r="B49" s="3"/>
-      <c r="C49" s="5"/>
+      <c r="A49" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="C49" s="5">
+        <v>1</v>
+      </c>
       <c r="D49" s="3"/>
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>
       <c r="G49" s="3" t="str">
         <f>IF(A49="","",Config!$B$2&amp;"?codigo="&amp;A49)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A048</v>
       </c>
     </row>
     <row r="50" spans="1:7">
-      <c r="A50" s="3"/>
-      <c r="B50" s="3"/>
-      <c r="C50" s="5"/>
+      <c r="A50" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="C50" s="5">
+        <v>1</v>
+      </c>
       <c r="D50" s="3"/>
       <c r="E50" s="3"/>
       <c r="F50" s="3"/>
       <c r="G50" s="3" t="str">
         <f>IF(A50="","",Config!$B$2&amp;"?codigo="&amp;A50)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A049</v>
       </c>
     </row>
     <row r="51" spans="1:7">
-      <c r="A51" s="3"/>
-      <c r="B51" s="3"/>
-      <c r="C51" s="5"/>
+      <c r="A51" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="C51" s="5">
+        <v>1</v>
+      </c>
       <c r="D51" s="3"/>
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
       <c r="G51" s="3" t="str">
         <f>IF(A51="","",Config!$B$2&amp;"?codigo="&amp;A51)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A050</v>
       </c>
     </row>
     <row r="52" spans="1:7">
-      <c r="A52" s="3"/>
-      <c r="B52" s="3"/>
-      <c r="C52" s="5"/>
+      <c r="A52" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="C52" s="5">
+        <v>1</v>
+      </c>
       <c r="D52" s="3"/>
       <c r="E52" s="3"/>
       <c r="F52" s="3"/>
       <c r="G52" s="3" t="str">
         <f>IF(A52="","",Config!$B$2&amp;"?codigo="&amp;A52)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A051</v>
       </c>
     </row>
     <row r="53" spans="1:7">
-      <c r="A53" s="3"/>
-      <c r="B53" s="3"/>
-      <c r="C53" s="5"/>
+      <c r="A53" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="C53" s="5">
+        <v>1</v>
+      </c>
       <c r="D53" s="3"/>
       <c r="E53" s="3"/>
       <c r="F53" s="3"/>
       <c r="G53" s="3" t="str">
         <f>IF(A53="","",Config!$B$2&amp;"?codigo="&amp;A53)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A052</v>
       </c>
     </row>
     <row r="54" spans="1:7">
-      <c r="A54" s="3"/>
-      <c r="B54" s="3"/>
-      <c r="C54" s="5"/>
+      <c r="A54" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="C54" s="5">
+        <v>1</v>
+      </c>
       <c r="D54" s="3"/>
       <c r="E54" s="3"/>
       <c r="F54" s="3"/>
       <c r="G54" s="3" t="str">
         <f>IF(A54="","",Config!$B$2&amp;"?codigo="&amp;A54)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A053</v>
       </c>
     </row>
     <row r="55" spans="1:7">
-      <c r="A55" s="3"/>
-      <c r="B55" s="3"/>
-      <c r="C55" s="5"/>
+      <c r="A55" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="C55" s="5">
+        <v>1</v>
+      </c>
       <c r="D55" s="3"/>
       <c r="E55" s="3"/>
       <c r="F55" s="3"/>
       <c r="G55" s="3" t="str">
         <f>IF(A55="","",Config!$B$2&amp;"?codigo="&amp;A55)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A054</v>
       </c>
     </row>
     <row r="56" spans="1:7">
-      <c r="A56" s="3"/>
-      <c r="B56" s="3"/>
-      <c r="C56" s="5"/>
+      <c r="A56" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="C56" s="5">
+        <v>1</v>
+      </c>
       <c r="D56" s="3"/>
       <c r="E56" s="3"/>
       <c r="F56" s="3"/>
       <c r="G56" s="3" t="str">
         <f>IF(A56="","",Config!$B$2&amp;"?codigo="&amp;A56)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A055</v>
       </c>
     </row>
     <row r="57" spans="1:7">
-      <c r="A57" s="3"/>
-      <c r="B57" s="3"/>
-      <c r="C57" s="5"/>
+      <c r="A57" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="C57" s="5">
+        <v>1</v>
+      </c>
       <c r="D57" s="3"/>
       <c r="E57" s="3"/>
       <c r="F57" s="3"/>
       <c r="G57" s="3" t="str">
         <f>IF(A57="","",Config!$B$2&amp;"?codigo="&amp;A57)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A056</v>
       </c>
     </row>
     <row r="58" spans="1:7">
-      <c r="A58" s="3"/>
-      <c r="B58" s="3"/>
-      <c r="C58" s="5"/>
+      <c r="A58" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="C58" s="5">
+        <v>1</v>
+      </c>
       <c r="D58" s="3"/>
       <c r="E58" s="3"/>
       <c r="F58" s="3"/>
       <c r="G58" s="3" t="str">
         <f>IF(A58="","",Config!$B$2&amp;"?codigo="&amp;A58)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A057</v>
       </c>
     </row>
     <row r="59" spans="1:7">
-      <c r="A59" s="3"/>
-      <c r="B59" s="3"/>
-      <c r="C59" s="5"/>
+      <c r="A59" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="C59" s="5">
+        <v>1</v>
+      </c>
       <c r="D59" s="3"/>
       <c r="E59" s="3"/>
       <c r="F59" s="3"/>
       <c r="G59" s="3" t="str">
         <f>IF(A59="","",Config!$B$2&amp;"?codigo="&amp;A59)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A058</v>
       </c>
     </row>
     <row r="60" spans="1:7">
-      <c r="A60" s="3"/>
-      <c r="B60" s="3"/>
-      <c r="C60" s="5"/>
+      <c r="A60" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="C60" s="5">
+        <v>1</v>
+      </c>
       <c r="D60" s="3"/>
       <c r="E60" s="3"/>
       <c r="F60" s="3"/>
       <c r="G60" s="3" t="str">
         <f>IF(A60="","",Config!$B$2&amp;"?codigo="&amp;A60)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A059</v>
       </c>
     </row>
     <row r="61" spans="1:7">
-      <c r="A61" s="3"/>
-      <c r="B61" s="3"/>
-      <c r="C61" s="5"/>
+      <c r="A61" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="C61" s="5">
+        <v>1</v>
+      </c>
       <c r="D61" s="3"/>
       <c r="E61" s="3"/>
       <c r="F61" s="3"/>
       <c r="G61" s="3" t="str">
         <f>IF(A61="","",Config!$B$2&amp;"?codigo="&amp;A61)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A060</v>
       </c>
     </row>
     <row r="62" spans="1:7">
-      <c r="A62" s="3"/>
-      <c r="B62" s="3"/>
-      <c r="C62" s="5"/>
+      <c r="A62" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="C62" s="5">
+        <v>1</v>
+      </c>
       <c r="D62" s="3"/>
       <c r="E62" s="3"/>
       <c r="F62" s="3"/>
       <c r="G62" s="3" t="str">
         <f>IF(A62="","",Config!$B$2&amp;"?codigo="&amp;A62)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A061</v>
       </c>
     </row>
     <row r="63" spans="1:7">
-      <c r="A63" s="3"/>
-      <c r="B63" s="3"/>
-      <c r="C63" s="5"/>
+      <c r="A63" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="C63" s="5">
+        <v>2</v>
+      </c>
       <c r="D63" s="3"/>
       <c r="E63" s="3"/>
       <c r="F63" s="3"/>
       <c r="G63" s="3" t="str">
         <f>IF(A63="","",Config!$B$2&amp;"?codigo="&amp;A63)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A062</v>
       </c>
     </row>
     <row r="64" spans="1:7">
-      <c r="A64" s="3"/>
-      <c r="B64" s="3"/>
-      <c r="C64" s="5"/>
+      <c r="A64" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="C64" s="5">
+        <v>1</v>
+      </c>
       <c r="D64" s="3"/>
       <c r="E64" s="3"/>
       <c r="F64" s="3"/>
       <c r="G64" s="3" t="str">
         <f>IF(A64="","",Config!$B$2&amp;"?codigo="&amp;A64)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A063</v>
       </c>
     </row>
     <row r="65" spans="1:7">
-      <c r="A65" s="3"/>
-      <c r="B65" s="3"/>
-      <c r="C65" s="5"/>
+      <c r="A65" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="C65" s="5">
+        <v>1</v>
+      </c>
       <c r="D65" s="3"/>
       <c r="E65" s="3"/>
       <c r="F65" s="3"/>
       <c r="G65" s="3" t="str">
         <f>IF(A65="","",Config!$B$2&amp;"?codigo="&amp;A65)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A064</v>
       </c>
     </row>
     <row r="66" spans="1:7">
-      <c r="A66" s="3"/>
-      <c r="B66" s="3"/>
-      <c r="C66" s="5"/>
+      <c r="A66" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="C66" s="5">
+        <v>1</v>
+      </c>
       <c r="D66" s="3"/>
       <c r="E66" s="3"/>
       <c r="F66" s="3"/>
       <c r="G66" s="3" t="str">
         <f>IF(A66="","",Config!$B$2&amp;"?codigo="&amp;A66)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A065</v>
       </c>
     </row>
     <row r="67" spans="1:7">
       <c r="A67" s="3"/>
-      <c r="B67" s="3"/>
-      <c r="C67" s="5"/>
       <c r="D67" s="3"/>
       <c r="E67" s="3"/>
       <c r="F67" s="3"/>
@@ -1422,8 +2095,6 @@
     </row>
     <row r="68" spans="1:7">
       <c r="A68" s="3"/>
-      <c r="B68" s="3"/>
-      <c r="C68" s="5"/>
       <c r="D68" s="3"/>
       <c r="E68" s="3"/>
       <c r="F68" s="3"/>
@@ -1434,8 +2105,6 @@
     </row>
     <row r="69" spans="1:7">
       <c r="A69" s="3"/>
-      <c r="B69" s="3"/>
-      <c r="C69" s="5"/>
       <c r="D69" s="3"/>
       <c r="E69" s="3"/>
       <c r="F69" s="3"/>
@@ -1446,8 +2115,6 @@
     </row>
     <row r="70" spans="1:7">
       <c r="A70" s="3"/>
-      <c r="B70" s="3"/>
-      <c r="C70" s="5"/>
       <c r="D70" s="3"/>
       <c r="E70" s="3"/>
       <c r="F70" s="3"/>
@@ -1458,8 +2125,6 @@
     </row>
     <row r="71" spans="1:7">
       <c r="A71" s="3"/>
-      <c r="B71" s="3"/>
-      <c r="C71" s="5"/>
       <c r="D71" s="3"/>
       <c r="E71" s="3"/>
       <c r="F71" s="3"/>
@@ -1470,8 +2135,6 @@
     </row>
     <row r="72" spans="1:7">
       <c r="A72" s="3"/>
-      <c r="B72" s="3"/>
-      <c r="C72" s="5"/>
       <c r="D72" s="3"/>
       <c r="E72" s="3"/>
       <c r="F72" s="3"/>
@@ -1482,8 +2145,6 @@
     </row>
     <row r="73" spans="1:7">
       <c r="A73" s="3"/>
-      <c r="B73" s="3"/>
-      <c r="C73" s="5"/>
       <c r="D73" s="3"/>
       <c r="E73" s="3"/>
       <c r="F73" s="3"/>
@@ -2423,19 +3084,22 @@
       <formula>AND(A2&lt;&gt;"",COUNTIF($A:$A,A2)&gt;1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C150">
+  <conditionalFormatting sqref="C2:C16 C74:C150 C21:C66">
     <cfRule type="expression" dxfId="0" priority="2">
       <formula>AND(C2&lt;&gt;"",C2&lt;1)</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="C2:C150" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation sqref="C2:C16 C21:C66 C74:C150" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>1</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="H9" r:id="rId1" xr:uid="{84750D8D-EB1D-4B48-BB12-E4CD89662A99}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -2471,7 +3135,7 @@
         <v>16</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>72</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3" spans="1:2">

</xml_diff>

<commit_message>
Corrige estructura de page e itinerario
</commit_message>
<xml_diff>
--- a/plantilla_invitados_xv_sandra_alicia.xlsx
+++ b/plantilla_invitados_xv_sandra_alicia.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\XVSandra\xvsandra\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD1B3DAC-2531-40F7-B393-00EE288A46D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5C8894E-A832-44CE-9D4A-D6F0D043BEFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="181">
   <si>
     <t>codigo</t>
   </si>
@@ -403,6 +403,12 @@
     <t>A065</t>
   </si>
   <si>
+    <t>A066</t>
+  </si>
+  <si>
+    <t>A067</t>
+  </si>
+  <si>
     <t>https://xvsandra.vercel.app/</t>
   </si>
   <si>
@@ -566,6 +572,12 @@
   </si>
   <si>
     <t>Gonzalo y Silvia Rosales</t>
+  </si>
+  <si>
+    <t>Alondra Menchaca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abby y Richy </t>
   </si>
 </sst>
 </file>
@@ -880,7 +892,7 @@
         <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -888,7 +900,7 @@
         <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C2">
         <v>2</v>
@@ -1040,7 +1052,7 @@
         <v>https://xvsandra.vercel.app/?codigo=A008</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -1162,7 +1174,7 @@
         <v>71</v>
       </c>
       <c r="B16" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C16">
         <v>2</v>
@@ -1182,7 +1194,7 @@
         <v>72</v>
       </c>
       <c r="B17" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C17">
         <v>2</v>
@@ -1202,7 +1214,7 @@
         <v>73</v>
       </c>
       <c r="B18" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C18">
         <v>2</v>
@@ -1222,7 +1234,7 @@
         <v>74</v>
       </c>
       <c r="B19" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C19">
         <v>1</v>
@@ -1242,7 +1254,7 @@
         <v>75</v>
       </c>
       <c r="B20" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C20">
         <v>2</v>
@@ -1260,7 +1272,7 @@
         <v>76</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C21" s="5">
         <v>1</v>
@@ -1278,7 +1290,7 @@
         <v>77</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C22" s="5">
         <v>1</v>
@@ -1296,7 +1308,7 @@
         <v>78</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C23" s="5">
         <v>1</v>
@@ -1314,7 +1326,7 @@
         <v>79</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C24" s="5">
         <v>1</v>
@@ -1332,7 +1344,7 @@
         <v>80</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C25" s="5">
         <v>1</v>
@@ -1350,7 +1362,7 @@
         <v>81</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C26" s="5">
         <v>1</v>
@@ -1368,7 +1380,7 @@
         <v>82</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C27" s="5">
         <v>1</v>
@@ -1386,7 +1398,7 @@
         <v>83</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C28" s="5">
         <v>1</v>
@@ -1404,7 +1416,7 @@
         <v>84</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C29" s="5">
         <v>1</v>
@@ -1422,7 +1434,7 @@
         <v>85</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C30" s="5">
         <v>1</v>
@@ -1440,7 +1452,7 @@
         <v>86</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C31" s="5">
         <v>1</v>
@@ -1458,7 +1470,7 @@
         <v>87</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C32" s="5">
         <v>1</v>
@@ -1476,7 +1488,7 @@
         <v>88</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C33" s="5">
         <v>1</v>
@@ -1494,7 +1506,7 @@
         <v>89</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C34" s="5">
         <v>1</v>
@@ -1512,7 +1524,7 @@
         <v>90</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C35" s="5">
         <v>1</v>
@@ -1530,7 +1542,7 @@
         <v>91</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C36" s="5">
         <v>1</v>
@@ -1548,7 +1560,7 @@
         <v>92</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C37" s="5">
         <v>1</v>
@@ -1566,7 +1578,7 @@
         <v>93</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C38" s="5">
         <v>1</v>
@@ -1584,7 +1596,7 @@
         <v>94</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C39" s="5">
         <v>1</v>
@@ -1602,7 +1614,7 @@
         <v>95</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C40" s="5">
         <v>1</v>
@@ -1620,7 +1632,7 @@
         <v>96</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C41" s="5">
         <v>1</v>
@@ -1638,7 +1650,7 @@
         <v>97</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C42" s="5">
         <v>1</v>
@@ -1656,7 +1668,7 @@
         <v>98</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C43" s="5">
         <v>2</v>
@@ -1674,7 +1686,7 @@
         <v>99</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C44" s="5">
         <v>1</v>
@@ -1692,7 +1704,7 @@
         <v>100</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C45" s="5">
         <v>1</v>
@@ -1710,7 +1722,7 @@
         <v>101</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C46" s="5">
         <v>1</v>
@@ -1728,7 +1740,7 @@
         <v>102</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C47" s="5">
         <v>1</v>
@@ -1746,7 +1758,7 @@
         <v>103</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C48" s="5">
         <v>1</v>
@@ -1764,7 +1776,7 @@
         <v>104</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C49" s="5">
         <v>1</v>
@@ -1782,7 +1794,7 @@
         <v>105</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C50" s="5">
         <v>1</v>
@@ -1800,7 +1812,7 @@
         <v>106</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C51" s="5">
         <v>1</v>
@@ -1818,7 +1830,7 @@
         <v>107</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C52" s="5">
         <v>1</v>
@@ -1836,7 +1848,7 @@
         <v>108</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C53" s="5">
         <v>1</v>
@@ -1854,7 +1866,7 @@
         <v>109</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C54" s="5">
         <v>1</v>
@@ -1872,7 +1884,7 @@
         <v>110</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C55" s="5">
         <v>1</v>
@@ -1890,7 +1902,7 @@
         <v>111</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C56" s="5">
         <v>1</v>
@@ -1908,7 +1920,7 @@
         <v>112</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C57" s="5">
         <v>1</v>
@@ -1926,7 +1938,7 @@
         <v>113</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C58" s="5">
         <v>1</v>
@@ -1944,7 +1956,7 @@
         <v>114</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C59" s="5">
         <v>1</v>
@@ -1962,7 +1974,7 @@
         <v>115</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C60" s="5">
         <v>1</v>
@@ -1980,7 +1992,7 @@
         <v>116</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C61" s="5">
         <v>1</v>
@@ -1998,7 +2010,7 @@
         <v>117</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C62" s="5">
         <v>1</v>
@@ -2016,7 +2028,7 @@
         <v>118</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C63" s="5">
         <v>2</v>
@@ -2034,7 +2046,7 @@
         <v>119</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C64" s="5">
         <v>1</v>
@@ -2052,7 +2064,7 @@
         <v>120</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C65" s="5">
         <v>1</v>
@@ -2070,7 +2082,7 @@
         <v>121</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C66" s="5">
         <v>1</v>
@@ -2084,23 +2096,41 @@
       </c>
     </row>
     <row r="67" spans="1:7">
-      <c r="A67" s="3"/>
+      <c r="A67" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B67" t="s">
+        <v>179</v>
+      </c>
+      <c r="C67">
+        <v>1</v>
+      </c>
       <c r="D67" s="3"/>
       <c r="E67" s="3"/>
       <c r="F67" s="3"/>
       <c r="G67" s="3" t="str">
         <f>IF(A67="","",Config!$B$2&amp;"?codigo="&amp;A67)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A066</v>
       </c>
     </row>
     <row r="68" spans="1:7">
-      <c r="A68" s="3"/>
-      <c r="D68" s="3"/>
+      <c r="A68" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B68" t="s">
+        <v>180</v>
+      </c>
+      <c r="C68">
+        <v>2</v>
+      </c>
+      <c r="D68" s="3">
+        <v>4422383550</v>
+      </c>
       <c r="E68" s="3"/>
       <c r="F68" s="3"/>
       <c r="G68" s="3" t="str">
         <f>IF(A68="","",Config!$B$2&amp;"?codigo="&amp;A68)</f>
-        <v/>
+        <v>https://xvsandra.vercel.app/?codigo=A067</v>
       </c>
     </row>
     <row r="69" spans="1:7">
@@ -3135,7 +3165,7 @@
         <v>16</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:2">

</xml_diff>